<commit_message>
Made some adjustments and added Persian Translation  by LLMs
</commit_message>
<xml_diff>
--- a/project1/reports/continue.dev/comparison prompt 1.xlsx
+++ b/project1/reports/continue.dev/comparison prompt 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Project Bachelor\project 1 small\reports\continue.dev\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Project Bachelor\unit-testing-with-genai\project1\reports\continue.dev\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4888A524-1E05-4C6F-B38C-D1B4FFE2A90E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19781F1F-BB0D-47DB-97E5-56387263FFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1035" windowWidth="29040" windowHeight="15720" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="7" xr2:uid="{5C34DE08-A12C-4EAA-A114-EBB56ADF1C7F}"/>
   </bookViews>
   <sheets>
     <sheet name="MyMath.checkSign(int)" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="104">
   <si>
     <t>testing a normal positive number</t>
   </si>
@@ -288,33 +288,9 @@
     <t>x is around  Integer.MAX_VALUE, y is large enough to cause overflow</t>
   </si>
   <si>
-    <t>general rule</t>
-  </si>
-  <si>
-    <t>Method names start with test</t>
-  </si>
-  <si>
-    <t>Boundary values checked</t>
-  </si>
-  <si>
-    <t>Private variables are used</t>
-  </si>
-  <si>
-    <t>Junit temporary storage is used</t>
-  </si>
-  <si>
-    <t>Edge cases tested</t>
-  </si>
-  <si>
-    <t>Methods have only a single assertion</t>
-  </si>
-  <si>
     <t>⚪️</t>
   </si>
   <si>
-    <t>Name of methods comply with what they test</t>
-  </si>
-  <si>
     <t>Qwen 3 Coder 30b</t>
   </si>
   <si>
@@ -355,6 +331,33 @@
   </si>
   <si>
     <t>indicating test is unnecessary in my opinion</t>
+  </si>
+  <si>
+    <t>قانون عمومی</t>
+  </si>
+  <si>
+    <t>نام آزمون ها مشخص می کند که چه چیزی تست می شود.</t>
+  </si>
+  <si>
+    <t>نام آزمون ها با test شروع می شود.</t>
+  </si>
+  <si>
+    <t>متغیر های خصوصی استفاده شده است.</t>
+  </si>
+  <si>
+    <t>مقادیر مرزی مورد آزمون قرار گرفته اند.</t>
+  </si>
+  <si>
+    <t>روش JUnit برای حافظه موقت استفاده شده است.</t>
+  </si>
+  <si>
+    <t>موارد حاشیه ای تست شده اند.</t>
+  </si>
+  <si>
+    <t>آزمون ها ها فقط یک assertion دارند.</t>
+  </si>
+  <si>
+    <t>در مخزن</t>
   </si>
 </sst>
 </file>
@@ -874,7 +877,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1140,7 +1143,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1190,7 +1193,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1508,7 +1511,7 @@
         <v>77</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1688,7 +1691,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B7" s="5">
         <v>0</v>
@@ -1723,7 +1726,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>24</v>
@@ -1793,13 +1796,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>78</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>12</v>
@@ -1828,7 +1831,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>24</v>
@@ -1933,13 +1936,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>12</v>
@@ -2003,10 +2006,10 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C16" s="5">
         <v>0</v>
@@ -2038,13 +2041,13 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B17" s="5">
         <v>0</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>12</v>
@@ -2093,7 +2096,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
@@ -2117,7 +2120,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2484,7 +2487,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2707,7 +2710,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -3249,7 +3252,7 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -3283,7 +3286,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
@@ -3524,22 +3527,22 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.140625" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="8" max="8" width="18.42578125" customWidth="1"/>
-    <col min="9" max="9" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>103</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>72</v>
@@ -3560,12 +3563,12 @@
         <v>77</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
@@ -3594,7 +3597,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
@@ -3623,7 +3626,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -3652,7 +3655,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>12</v>
@@ -3681,7 +3684,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>12</v>
@@ -3710,7 +3713,7 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
@@ -3739,7 +3742,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
@@ -3748,10 +3751,10 @@
         <v>12</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>11</v>
@@ -3763,7 +3766,7 @@
         <v>11</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>